<commit_message>
Add LCSC properties to components and exclude specific through-hole parts from BOM
</commit_message>
<xml_diff>
--- a/BOM_PCBWay.xlsx
+++ b/BOM_PCBWay.xlsx
@@ -132,7 +132,7 @@
     <t xml:space="preserve">C1</t>
   </si>
   <si>
-    <t xml:space="preserve">GRM31CR71H104KA01L</t>
+    <t xml:space="preserve">GRM31MR71H104KA01L</t>
   </si>
   <si>
     <t xml:space="preserve">100nF (Unpolarized capacitor)</t>
@@ -146,7 +146,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,6 +211,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -302,100 +308,104 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -482,9 +492,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>666000</xdr:colOff>
+      <xdr:colOff>665640</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>156240</xdr:rowOff>
+      <xdr:rowOff>155880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -498,7 +508,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="209520"/>
-          <a:ext cx="1365480" cy="375480"/>
+          <a:ext cx="1365120" cy="375120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -701,7 +711,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.38"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="74.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="58.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.85"/>
@@ -952,7 +962,7 @@
       <c r="D13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F13" s="8" t="s">
@@ -1006,92 +1016,92 @@
       <c r="J16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="20"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-    </row>
-    <row r="26" s="23" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+    </row>
+    <row r="26" s="24" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>